<commit_message>
Sql fájl insert into javítása
</commit_message>
<xml_diff>
--- a/utvonalak.xlsx
+++ b/utvonalak.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Plane\Desktop\szakmai_projekt\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Plane\Desktop\ItBeeZ_Github_Szakmai\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4DD48F96-FAAF-4F9D-9D30-47FE3B3AD535}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E333E30-D9B2-4566-97BB-2720DE7A72F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7CDF2E19-D32D-403D-B891-900F3CE22FEE}"/>
   </bookViews>
@@ -373,12 +373,24 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC00000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -393,10 +405,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normál" xfId="0" builtinId="0"/>
@@ -717,147 +733,153 @@
     <col min="1" max="1" width="26" style="2" customWidth="1"/>
     <col min="2" max="2" width="41" style="1" customWidth="1"/>
     <col min="3" max="3" width="19.21875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="31.77734375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="45.77734375" style="1" customWidth="1"/>
     <col min="5" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
+      <c r="C1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D2" s="1" t="s">
+      <c r="C2" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" s="6" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D4" s="6" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="D5" s="4" t="s">
         <v>5</v>
       </c>
     </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="3"/>
+      <c r="B6" s="4"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+    </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D7" s="1" t="s">
+      <c r="C7" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D7" s="4" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C8" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D8" s="1" t="s">
+      <c r="C8" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D8" s="4" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C9" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="D9" s="4" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="D10" s="4" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C11" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="D11" s="4" t="s">
         <v>15</v>
       </c>
     </row>
@@ -1520,44 +1542,44 @@
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A69" s="2" t="s">
+      <c r="A69" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="B69" s="1" t="s">
+      <c r="B69" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="C69" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D69" s="1" t="s">
+      <c r="C69" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D69" s="4" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A70" s="2" t="s">
+      <c r="A70" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="B70" s="1" t="s">
+      <c r="B70" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="C70" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D70" s="1" t="s">
+      <c r="C70" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D70" s="4" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A71" s="2" t="s">
+      <c r="A71" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="B71" s="1" t="s">
+      <c r="B71" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="C71" s="1" t="s">
+      <c r="C71" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D71" s="1" t="s">
+      <c r="D71" s="4" t="s">
         <v>101</v>
       </c>
     </row>

</xml_diff>